<commit_message>
Correct moving-mass limiter gates
</commit_message>
<xml_diff>
--- a/results/analysis/moving_mass_gain_resweep/moving_mass_gain_resweep.xlsx
+++ b/results/analysis/moving_mass_gain_resweep/moving_mass_gain_resweep.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra2fdad699aec403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gain Ranking" sheetId="2" r:id="R590262ea35534e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="3" r:id="Rf261bb50bf594674"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Gates" sheetId="4" r:id="Ra199380843c14ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejections" sheetId="5" r:id="Rd0269fdc375f4c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" r:id="R4a04f88fd5c7487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Reaaec09ab46b44dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gain Ranking" sheetId="2" r:id="Rdcbdd6cb606641b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="3" r:id="Rb2aabe9abcee4f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Gates" sheetId="4" r:id="R5936a19774b14f35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limiter Diagnostics" sheetId="5" r:id="R6644eef6c0ec4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejections" sheetId="6" r:id="R8cef17b49d9a4878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="7" r:id="Reb5f0335af6a49bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,11 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0.00000"/>
     <x:numFmt numFmtId="201" formatCode="0.000000000"/>
     <x:numFmt numFmtId="202" formatCode="0.000000"/>
-    <x:numFmt numFmtId="203" formatCode="0.000%"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -87,7 +87,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="24">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -137,7 +137,6 @@
         </x:ext>
       </x:extLst>
     </x:xf>
-    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
@@ -166,9 +165,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GainRankingTable" displayName="GainRankingTable" ref="A1:N34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:N34"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GainRankingTable" displayName="GainRankingTable" ref="A1:O54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:O54"/>
+  <x:tableColumns count="15">
     <x:tableColumn id="1" name="Stage"/>
     <x:tableColumn id="2" name="Rank"/>
     <x:tableColumn id="3" name="Gain (m/Nm)"/>
@@ -182,21 +181,22 @@
     <x:tableColumn id="11" name="Mean vane TV (deg)"/>
     <x:tableColumn id="12" name="Mean mass RMS (m)"/>
     <x:tableColumn id="13" name="Mean mass travel (m)"/>
-    <x:tableColumn id="14" name="Worst symmetry"/>
+    <x:tableColumn id="14" name="Mean accel limiter duty %"/>
+    <x:tableColumn id="15" name="Worst symmetry"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComparisonTable" displayName="ComparisonTable" ref="A3:E18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:E18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComparisonTable" displayName="ComparisonTable" ref="A3:E25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:E25"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Metric"/>
     <x:tableColumn id="2" name="Gain 0 Vane-only"/>
     <x:tableColumn id="3" name="Old PR #20 0.1325"/>
     <x:tableColumn id="4" name="Selected"/>
-    <x:tableColumn id="5" name="Selected vs gain 0"/>
+    <x:tableColumn id="5" name="Selected minus gain 0"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -231,8 +231,32 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RejectionSummaryTable" displayName="RejectionSummaryTable" ref="A1:B4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:B4"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="LimiterDiagnosticsTable" displayName="LimiterDiagnosticsTable" ref="A3:O24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:O24"/>
+  <x:tableColumns count="15">
+    <x:tableColumn id="1" name="Scenario"/>
+    <x:tableColumn id="2" name="Controller set"/>
+    <x:tableColumn id="3" name="Rejected"/>
+    <x:tableColumn id="4" name="Command clip duty %"/>
+    <x:tableColumn id="5" name="Command clip longest s"/>
+    <x:tableColumn id="6" name="Rail contact duty %"/>
+    <x:tableColumn id="7" name="Rail contact longest s"/>
+    <x:tableColumn id="8" name="Rate limiter duty %"/>
+    <x:tableColumn id="9" name="Rate limiter longest s"/>
+    <x:tableColumn id="10" name="Accel limiter duty %"/>
+    <x:tableColumn id="11" name="Accel limiter longest s"/>
+    <x:tableColumn id="12" name="Actual max offset m"/>
+    <x:tableColumn id="13" name="Actual max rate m/s"/>
+    <x:tableColumn id="14" name="Actual max accel m/s²"/>
+    <x:tableColumn id="15" name="Reasons"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RejectionSummaryTable" displayName="RejectionSummaryTable" ref="A1:B6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:B6"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Rejection category"/>
     <x:tableColumn id="2" name="Candidate count"/>
@@ -486,19 +510,19 @@
         <x:v>0.09375</x:v>
       </x:c>
       <x:c r="D7" s="15" t="str">
-        <x:v>retain_gain_zero_valid_raw_score_rank1</x:v>
+        <x:v>adopt_valid_raw_score_rank1</x:v>
       </x:c>
       <x:c r="E7" s="16" t="n">
-        <x:v>1.5</x:v>
+        <x:v>0.5858400877649983</x:v>
       </x:c>
       <x:c r="F7" s="16" t="n">
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="G7" s="15" t="n">
-        <x:v>0</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="H7" s="15" t="n">
-        <x:v>29</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -517,7 +541,7 @@
         <x:v>0.021</x:v>
       </x:c>
       <x:c r="D9" s="19" t="str">
-        <x:v>Result: gain 0.00000 is the valid raw-score rank-1 candidate. Every nonzero tested gain is hard-rejected for Moving-mass saturation and/or acceleration-limit saturation. Moving-mass target and actual displacement therefore remain exactly zero for the adopted profile.</x:v>
+        <x:v>Result: gain 0.04150 is the valid raw-score rank-1 candidate. Normal Moving-mass limiter activity is recorded and penalized; only excessive duty/continuous duration or actual physical-limit violations are rejected. The selected profile passed every hard gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -573,7 +597,7 @@
         <x:v>Selected gain (m/Nm)</x:v>
       </x:c>
       <x:c r="B16" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0415</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -647,6 +671,9 @@
         <x:v>Mean mass travel (m)</x:v>
       </x:c>
       <x:c r="N1" s="10" t="str">
+        <x:v>Mean accel limiter duty %</x:v>
+      </x:c>
+      <x:c r="O1" s="10" t="str">
         <x:v>Worst symmetry</x:v>
       </x:c>
     </x:row>
@@ -689,6 +716,9 @@
       <x:c r="N2" s="21" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O2" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
@@ -698,7 +728,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.05</x:v>
       </x:c>
       <x:c r="D3" s="21" t="n">
         <x:v>7</x:v>
@@ -708,27 +738,30 @@
       </x:c>
       <x:c r="F3" s="21" t="str"/>
       <x:c r="G3" s="21" t="n">
-        <x:v>1.5</x:v>
+        <x:v>0.7589796823592732</x:v>
       </x:c>
       <x:c r="H3" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>0.4832517199660086</x:v>
       </x:c>
       <x:c r="I3" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5345654939496111</x:v>
       </x:c>
       <x:c r="J3" s="21" t="n">
-        <x:v>0.7324137788938853</x:v>
+        <x:v>0.5874687637500261</x:v>
       </x:c>
       <x:c r="K3" s="21" t="n">
-        <x:v>34.517019466703736</x:v>
+        <x:v>21.521822160330142</x:v>
       </x:c>
       <x:c r="L3" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0011338560397958026</x:v>
       </x:c>
       <x:c r="M3" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.03595660448683733</x:v>
       </x:c>
       <x:c r="N3" s="21" t="n">
+        <x:v>5.7857142857142865</x:v>
+      </x:c>
+      <x:c r="O3" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -736,7 +769,9 @@
       <x:c r="A4" t="str">
         <x:v>stage1_coarse</x:v>
       </x:c>
-      <x:c r="B4" t="str"/>
+      <x:c r="B4" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C4" s="21" t="n">
         <x:v>0.025</x:v>
       </x:c>
@@ -744,19 +779,17 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E4" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F4" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G4" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="str"/>
+      <x:c r="G4" s="21" t="n">
+        <x:v>1.0524913310625879</x:v>
       </x:c>
       <x:c r="H4" s="21" t="n">
-        <x:v>0.7066252342175213</x:v>
+        <x:v>0.7097502342175211</x:v>
       </x:c>
       <x:c r="I4" s="21" t="n">
-        <x:v>0.9752444579327862</x:v>
+        <x:v>0.9773694579327863</x:v>
       </x:c>
       <x:c r="J4" s="21" t="n">
         <x:v>0.5969576006359417</x:v>
@@ -771,6 +804,9 @@
         <x:v>0.019451165080231727</x:v>
       </x:c>
       <x:c r="N4" s="21" t="n">
+        <x:v>3.125</x:v>
+      </x:c>
+      <x:c r="O4" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -778,41 +814,44 @@
       <x:c r="A5" t="str">
         <x:v>stage1_coarse</x:v>
       </x:c>
-      <x:c r="B5" t="str"/>
+      <x:c r="B5" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C5" s="21" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.075</x:v>
       </x:c>
       <x:c r="D5" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E5" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F5" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G5" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="21" t="str"/>
+      <x:c r="G5" s="21" t="n">
+        <x:v>1.2537933910753518</x:v>
       </x:c>
       <x:c r="H5" s="21" t="n">
-        <x:v>0.47728743425172276</x:v>
+        <x:v>0.8498769166154798</x:v>
       </x:c>
       <x:c r="I5" s="21" t="n">
-        <x:v>0.527190493949611</x:v>
+        <x:v>1.4250291152838965</x:v>
       </x:c>
       <x:c r="J5" s="21" t="n">
-        <x:v>0.5874687637500261</x:v>
+        <x:v>0.6873889356742513</x:v>
       </x:c>
       <x:c r="K5" s="21" t="n">
-        <x:v>21.521822160330142</x:v>
+        <x:v>28.767204004840345</x:v>
       </x:c>
       <x:c r="L5" s="21" t="n">
-        <x:v>0.0011338560397958026</x:v>
+        <x:v>0.00208202550290569</x:v>
       </x:c>
       <x:c r="M5" s="21" t="n">
-        <x:v>0.03595660448683733</x:v>
+        <x:v>0.07495154535628075</x:v>
       </x:c>
       <x:c r="N5" s="21" t="n">
+        <x:v>11.982142857142856</x:v>
+      </x:c>
+      <x:c r="O5" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -820,41 +859,44 @@
       <x:c r="A6" t="str">
         <x:v>stage1_coarse</x:v>
       </x:c>
-      <x:c r="B6" t="str"/>
+      <x:c r="B6" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C6" s="21" t="n">
-        <x:v>0.075</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E6" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F6" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G6" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="21" t="str"/>
+      <x:c r="G6" s="21" t="n">
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="H6" s="21" t="n">
-        <x:v>0.8365792975678608</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I6" s="21" t="n">
-        <x:v>1.4162791152838965</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J6" s="21" t="n">
-        <x:v>0.6873889356742513</x:v>
+        <x:v>0.7324137788938853</x:v>
       </x:c>
       <x:c r="K6" s="21" t="n">
-        <x:v>28.767204004840345</x:v>
+        <x:v>34.517019466703736</x:v>
       </x:c>
       <x:c r="L6" s="21" t="n">
-        <x:v>0.00208202550290569</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="21" t="n">
-        <x:v>0.07495154535628075</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O6" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -873,16 +915,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F7" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_acceleration_limiter_duty</x:v>
       </x:c>
       <x:c r="G7" s="21" t="str">
         <x:v>inf</x:v>
       </x:c>
       <x:c r="H7" s="21" t="n">
-        <x:v>0.8429550574304073</x:v>
+        <x:v>0.8761693431446932</x:v>
       </x:c>
       <x:c r="I7" s="21" t="n">
-        <x:v>1.1966847972249097</x:v>
+        <x:v>1.2412472972249098</x:v>
       </x:c>
       <x:c r="J7" s="21" t="n">
         <x:v>0.873051512468919</x:v>
@@ -897,6 +939,9 @@
         <x:v>0.20109886460786744</x:v>
       </x:c>
       <x:c r="N7" s="21" t="n">
+        <x:v>28.815476190476193</x:v>
+      </x:c>
+      <x:c r="O7" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -915,16 +960,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F8" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="G8" s="21" t="str">
         <x:v>inf</x:v>
       </x:c>
       <x:c r="H8" s="21" t="n">
-        <x:v>2.215644507628517</x:v>
+        <x:v>2.344436174295184</x:v>
       </x:c>
       <x:c r="I8" s="21" t="n">
-        <x:v>2.576167838039456</x:v>
+        <x:v>2.7191261713727894</x:v>
       </x:c>
       <x:c r="J8" s="21" t="n">
         <x:v>1.7283888658478237</x:v>
@@ -939,6 +984,9 @@
         <x:v>0.6805598089286148</x:v>
       </x:c>
       <x:c r="N8" s="21" t="n">
+        <x:v>81.74999999999999</x:v>
+      </x:c>
+      <x:c r="O8" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -957,16 +1005,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="G9" s="21" t="str">
         <x:v>inf</x:v>
       </x:c>
       <x:c r="H9" s="21" t="n">
-        <x:v>2.4501458523318336</x:v>
+        <x:v>2.583979185665167</x:v>
       </x:c>
       <x:c r="I9" s="21" t="n">
-        <x:v>2.813935115137125</x:v>
+        <x:v>2.976685115137125</x:v>
       </x:c>
       <x:c r="J9" s="21" t="n">
         <x:v>1.8244210288332037</x:v>
@@ -981,6 +1029,9 @@
         <x:v>0.6996131934251938</x:v>
       </x:c>
       <x:c r="N9" s="21" t="n">
+        <x:v>82.23214285714286</x:v>
+      </x:c>
+      <x:c r="O9" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -999,16 +1050,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F10" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="G10" s="21" t="str">
         <x:v>inf</x:v>
       </x:c>
       <x:c r="H10" s="21" t="n">
-        <x:v>2.675592372559305</x:v>
+        <x:v>2.8158126106545436</x:v>
       </x:c>
       <x:c r="I10" s="21" t="n">
-        <x:v>3.200470671060463</x:v>
+        <x:v>3.356845671060463</x:v>
       </x:c>
       <x:c r="J10" s="21" t="n">
         <x:v>2.008300060332248</x:v>
@@ -1023,6 +1074,9 @@
         <x:v>0.7326494676154425</x:v>
       </x:c>
       <x:c r="N10" s="21" t="n">
+        <x:v>82.46428571428571</x:v>
+      </x:c>
+      <x:c r="O10" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1041,16 +1095,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="G11" s="21" t="str">
         <x:v>inf</x:v>
       </x:c>
       <x:c r="H11" s="21" t="n">
-        <x:v>3.209238198083042</x:v>
+        <x:v>3.370839388559232</x:v>
       </x:c>
       <x:c r="I11" s="21" t="n">
-        <x:v>3.263227958765976</x:v>
+        <x:v>3.425102958765976</x:v>
       </x:c>
       <x:c r="J11" s="21" t="n">
         <x:v>2.3508457227126063</x:v>
@@ -1065,6 +1119,9 @@
         <x:v>0.8455994906879736</x:v>
       </x:c>
       <x:c r="N11" s="21" t="n">
+        <x:v>92.30952380952381</x:v>
+      </x:c>
+      <x:c r="O11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1083,16 +1140,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F12" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit; second_acceleration_lobe_after_full_pause</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration; second_acceleration_lobe_after_full_pause</x:v>
       </x:c>
       <x:c r="G12" s="21" t="str">
         <x:v>inf</x:v>
       </x:c>
       <x:c r="H12" s="21" t="n">
-        <x:v>3.5127391256875797</x:v>
+        <x:v>3.6839950780685315</x:v>
       </x:c>
       <x:c r="I12" s="21" t="n">
-        <x:v>3.5551216829965258</x:v>
+        <x:v>3.7302058394340794</x:v>
       </x:c>
       <x:c r="J12" s="21" t="n">
         <x:v>2.553544052667369</x:v>
@@ -1107,6 +1164,9 @@
         <x:v>0.8943128189059014</x:v>
       </x:c>
       <x:c r="N12" s="21" t="n">
+        <x:v>93.60119047619048</x:v>
+      </x:c>
+      <x:c r="O12" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1118,7 +1178,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C13" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0425</x:v>
       </x:c>
       <x:c r="D13" s="21" t="n">
         <x:v>7</x:v>
@@ -1128,27 +1188,30 @@
       </x:c>
       <x:c r="F13" s="21" t="str"/>
       <x:c r="G13" s="21" t="n">
-        <x:v>1.5</x:v>
+        <x:v>0.5879499406370574</x:v>
       </x:c>
       <x:c r="H13" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>0.4153507439082819</x:v>
       </x:c>
       <x:c r="I13" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>0.6329659406051644</x:v>
       </x:c>
       <x:c r="J13" s="21" t="n">
-        <x:v>0.7324137788938853</x:v>
+        <x:v>0.5785728446559552</x:v>
       </x:c>
       <x:c r="K13" s="21" t="n">
-        <x:v>34.517019466703736</x:v>
+        <x:v>20.598195413255667</x:v>
       </x:c>
       <x:c r="L13" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0009543818996144423</x:v>
       </x:c>
       <x:c r="M13" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.029398426514506637</x:v>
       </x:c>
       <x:c r="N13" s="21" t="n">
+        <x:v>4.845238095238096</x:v>
+      </x:c>
+      <x:c r="O13" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1156,41 +1219,44 @@
       <x:c r="A14" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B14" t="str"/>
+      <x:c r="B14" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C14" s="21" t="n">
-        <x:v>0.0025</x:v>
+        <x:v>0.0475</x:v>
       </x:c>
       <x:c r="D14" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E14" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F14" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G14" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="21" t="str"/>
+      <x:c r="G14" s="21" t="n">
+        <x:v>0.6231404368575117</x:v>
       </x:c>
       <x:c r="H14" s="21" t="n">
-        <x:v>1.0270475665765908</x:v>
+        <x:v>0.3903972793717462</x:v>
       </x:c>
       <x:c r="I14" s="21" t="n">
-        <x:v>1.0666528404242814</x:v>
+        <x:v>0.7833822924878484</x:v>
       </x:c>
       <x:c r="J14" s="21" t="n">
-        <x:v>0.7215036643063957</x:v>
+        <x:v>0.5848557285559549</x:v>
       </x:c>
       <x:c r="K14" s="21" t="n">
-        <x:v>33.80561276626928</x:v>
+        <x:v>21.173191272766253</x:v>
       </x:c>
       <x:c r="L14" s="21" t="n">
-        <x:v>0.00009942141985853976</x:v>
+        <x:v>0.0010615376969566204</x:v>
       </x:c>
       <x:c r="M14" s="21" t="n">
-        <x:v>0.004861485797871268</x:v>
+        <x:v>0.03348034548688624</x:v>
       </x:c>
       <x:c r="N14" s="21" t="n">
+        <x:v>5.136904761904762</x:v>
+      </x:c>
+      <x:c r="O14" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1198,41 +1264,44 @@
       <x:c r="A15" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B15" t="str"/>
+      <x:c r="B15" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C15" s="21" t="n">
-        <x:v>0.005</x:v>
+        <x:v>0.045</x:v>
       </x:c>
       <x:c r="D15" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E15" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F15" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G15" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="21" t="str"/>
+      <x:c r="G15" s="21" t="n">
+        <x:v>0.6688585407275436</x:v>
       </x:c>
       <x:c r="H15" s="21" t="n">
-        <x:v>1.0506585021333839</x:v>
+        <x:v>0.4609825115381697</x:v>
       </x:c>
       <x:c r="I15" s="21" t="n">
-        <x:v>1.0797285385370963</x:v>
+        <x:v>0.5469503295641454</x:v>
       </x:c>
       <x:c r="J15" s="21" t="n">
-        <x:v>0.7144184093790183</x:v>
+        <x:v>0.5829696426603963</x:v>
       </x:c>
       <x:c r="K15" s="21" t="n">
-        <x:v>32.543069872365784</x:v>
+        <x:v>20.671351753002295</x:v>
       </x:c>
       <x:c r="L15" s="21" t="n">
-        <x:v>0.00018843105190779883</x:v>
+        <x:v>0.0010099097878908904</x:v>
       </x:c>
       <x:c r="M15" s="21" t="n">
-        <x:v>0.008829584942994512</x:v>
+        <x:v>0.030771802061914478</x:v>
       </x:c>
       <x:c r="N15" s="21" t="n">
+        <x:v>4.916666666666666</x:v>
+      </x:c>
+      <x:c r="O15" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1240,41 +1309,44 @@
       <x:c r="A16" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B16" t="str"/>
+      <x:c r="B16" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C16" s="21" t="n">
-        <x:v>0.0075</x:v>
+        <x:v>0.035</x:v>
       </x:c>
       <x:c r="D16" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E16" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F16" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G16" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="21" t="str"/>
+      <x:c r="G16" s="21" t="n">
+        <x:v>0.6857317802655519</x:v>
       </x:c>
       <x:c r="H16" s="21" t="n">
-        <x:v>1.0587259801632236</x:v>
+        <x:v>0.46652666320755853</x:v>
       </x:c>
       <x:c r="I16" s="21" t="n">
-        <x:v>1.1020001221947773</x:v>
+        <x:v>0.6753024626855436</x:v>
       </x:c>
       <x:c r="J16" s="21" t="n">
-        <x:v>0.7054448050483036</x:v>
+        <x:v>0.5830587093945818</x:v>
       </x:c>
       <x:c r="K16" s="21" t="n">
-        <x:v>31.808039497250256</x:v>
+        <x:v>20.29955767967368</x:v>
       </x:c>
       <x:c r="L16" s="21" t="n">
-        <x:v>0.00026354256523693226</x:v>
+        <x:v>0.0007925741900682977</x:v>
       </x:c>
       <x:c r="M16" s="21" t="n">
-        <x:v>0.012284549438691674</x:v>
+        <x:v>0.02429958274077779</x:v>
       </x:c>
       <x:c r="N16" s="21" t="n">
+        <x:v>4.035714285714286</x:v>
+      </x:c>
+      <x:c r="O16" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1282,41 +1354,44 @@
       <x:c r="A17" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B17" t="str"/>
+      <x:c r="B17" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C17" s="21" t="n">
-        <x:v>0.01</x:v>
+        <x:v>0.0525</x:v>
       </x:c>
       <x:c r="D17" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E17" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F17" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G17" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="21" t="str"/>
+      <x:c r="G17" s="21" t="n">
+        <x:v>0.7471622146356975</x:v>
       </x:c>
       <x:c r="H17" s="21" t="n">
-        <x:v>0.949128935028396</x:v>
+        <x:v>0.47823955866387463</x:v>
       </x:c>
       <x:c r="I17" s="21" t="n">
-        <x:v>0.9867394532725388</x:v>
+        <x:v>0.6460990481538518</x:v>
       </x:c>
       <x:c r="J17" s="21" t="n">
-        <x:v>0.6955050301985759</x:v>
+        <x:v>0.5913876431981395</x:v>
       </x:c>
       <x:c r="K17" s="21" t="n">
-        <x:v>31.106651947829004</x:v>
+        <x:v>21.91047602030281</x:v>
       </x:c>
       <x:c r="L17" s="21" t="n">
-        <x:v>0.0003315053397496943</x:v>
+        <x:v>0.001197966300710091</x:v>
       </x:c>
       <x:c r="M17" s="21" t="n">
-        <x:v>0.015276522377715715</x:v>
+        <x:v>0.038486909992846756</x:v>
       </x:c>
       <x:c r="N17" s="21" t="n">
+        <x:v>5.970238095238096</x:v>
+      </x:c>
+      <x:c r="O17" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1324,41 +1399,44 @@
       <x:c r="A18" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B18" t="str"/>
+      <x:c r="B18" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C18" s="21" t="n">
-        <x:v>0.0125</x:v>
+        <x:v>0.05</x:v>
       </x:c>
       <x:c r="D18" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E18" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F18" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G18" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="21" t="str"/>
+      <x:c r="G18" s="21" t="n">
+        <x:v>0.7589796823592732</x:v>
       </x:c>
       <x:c r="H18" s="21" t="n">
-        <x:v>0.9520639603710169</x:v>
+        <x:v>0.4832517199660086</x:v>
       </x:c>
       <x:c r="I18" s="21" t="n">
-        <x:v>0.9827320108735196</x:v>
+        <x:v>0.5345654939496111</x:v>
       </x:c>
       <x:c r="J18" s="21" t="n">
-        <x:v>0.6856930204018459</x:v>
+        <x:v>0.5874687637500261</x:v>
       </x:c>
       <x:c r="K18" s="21" t="n">
-        <x:v>30.449286475939125</x:v>
+        <x:v>21.521822160330142</x:v>
       </x:c>
       <x:c r="L18" s="21" t="n">
-        <x:v>0.0003970246599184876</x:v>
+        <x:v>0.0011338560397958026</x:v>
       </x:c>
       <x:c r="M18" s="21" t="n">
-        <x:v>0.018067108596170493</x:v>
+        <x:v>0.03595660448683733</x:v>
       </x:c>
       <x:c r="N18" s="21" t="n">
+        <x:v>5.7857142857142865</x:v>
+      </x:c>
+      <x:c r="O18" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1366,41 +1444,44 @@
       <x:c r="A19" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B19" t="str"/>
+      <x:c r="B19" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C19" s="21" t="n">
-        <x:v>0.015</x:v>
+        <x:v>0.04</x:v>
       </x:c>
       <x:c r="D19" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E19" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F19" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G19" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="21" t="str"/>
+      <x:c r="G19" s="21" t="n">
+        <x:v>0.8313096468709749</x:v>
       </x:c>
       <x:c r="H19" s="21" t="n">
-        <x:v>0.9678655494063341</x:v>
+        <x:v>0.5462156895750908</x:v>
       </x:c>
       <x:c r="I19" s="21" t="n">
-        <x:v>1.0304341494299125</x:v>
+        <x:v>0.9412516624258085</x:v>
       </x:c>
       <x:c r="J19" s="21" t="n">
-        <x:v>0.675139046111634</x:v>
+        <x:v>0.5782834299435242</x:v>
       </x:c>
       <x:c r="K19" s="21" t="n">
-        <x:v>28.9614563694579</x:v>
+        <x:v>20.33680183680493</x:v>
       </x:c>
       <x:c r="L19" s="21" t="n">
-        <x:v>0.00045879359708805124</x:v>
+        <x:v>0.0009063263727419075</x:v>
       </x:c>
       <x:c r="M19" s="21" t="n">
-        <x:v>0.019859446832295923</x:v>
+        <x:v>0.027300113650715264</x:v>
       </x:c>
       <x:c r="N19" s="21" t="n">
+        <x:v>4.553571428571429</x:v>
+      </x:c>
+      <x:c r="O19" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1408,41 +1489,44 @@
       <x:c r="A20" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B20" t="str"/>
+      <x:c r="B20" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C20" s="21" t="n">
-        <x:v>0.0175</x:v>
+        <x:v>0.0325</x:v>
       </x:c>
       <x:c r="D20" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E20" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F20" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G20" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F20" s="21" t="str"/>
+      <x:c r="G20" s="21" t="n">
+        <x:v>0.8338953257567154</x:v>
       </x:c>
       <x:c r="H20" s="21" t="n">
-        <x:v>0.7551654323670535</x:v>
+        <x:v>0.5508310068403522</x:v>
       </x:c>
       <x:c r="I20" s="21" t="n">
-        <x:v>0.9787798121233477</x:v>
+        <x:v>0.7597545599966085</x:v>
       </x:c>
       <x:c r="J20" s="21" t="n">
-        <x:v>0.6434867270062382</x:v>
+        <x:v>0.5882869671770532</x:v>
       </x:c>
       <x:c r="K20" s="21" t="n">
-        <x:v>25.571734842922837</x:v>
+        <x:v>20.209024885463844</x:v>
       </x:c>
       <x:c r="L20" s="21" t="n">
-        <x:v>0.00048334149758123314</x:v>
+        <x:v>0.0007490442881841724</x:v>
       </x:c>
       <x:c r="M20" s="21" t="n">
-        <x:v>0.019006168693760234</x:v>
+        <x:v>0.022638968964258255</x:v>
       </x:c>
       <x:c r="N20" s="21" t="n">
+        <x:v>4.065476190476191</x:v>
+      </x:c>
+      <x:c r="O20" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1450,41 +1534,44 @@
       <x:c r="A21" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B21" t="str"/>
+      <x:c r="B21" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C21" s="21" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.0375</x:v>
       </x:c>
       <x:c r="D21" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E21" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F21" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G21" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="21" t="str"/>
+      <x:c r="G21" s="21" t="n">
+        <x:v>0.990114187197696</x:v>
       </x:c>
       <x:c r="H21" s="21" t="n">
-        <x:v>0.6001646528893195</x:v>
+        <x:v>0.634110600555118</x:v>
       </x:c>
       <x:c r="I21" s="21" t="n">
-        <x:v>1.0042437777450326</x:v>
+        <x:v>0.9084012417761826</x:v>
       </x:c>
       <x:c r="J21" s="21" t="n">
-        <x:v>0.6207556226106367</x:v>
+        <x:v>0.5820238621281989</x:v>
       </x:c>
       <x:c r="K21" s="21" t="n">
-        <x:v>23.45890809707205</x:v>
+        <x:v>20.308352579412112</x:v>
       </x:c>
       <x:c r="L21" s="21" t="n">
-        <x:v>0.0005104514029752476</x:v>
+        <x:v>0.0008576574770892432</x:v>
       </x:c>
       <x:c r="M21" s="21" t="n">
-        <x:v>0.018732146953448738</x:v>
+        <x:v>0.02579059223383672</x:v>
       </x:c>
       <x:c r="N21" s="21" t="n">
+        <x:v>4.035714285714286</x:v>
+      </x:c>
+      <x:c r="O21" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1492,41 +1579,44 @@
       <x:c r="A22" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B22" t="str"/>
+      <x:c r="B22" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C22" s="21" t="n">
-        <x:v>0.0225</x:v>
+        <x:v>0.055</x:v>
       </x:c>
       <x:c r="D22" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E22" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F22" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G22" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="21" t="str"/>
+      <x:c r="G22" s="21" t="n">
+        <x:v>0.9903951627819696</x:v>
       </x:c>
       <x:c r="H22" s="21" t="n">
-        <x:v>1.1372119020473235</x:v>
+        <x:v>0.6101781422902424</x:v>
       </x:c>
       <x:c r="I22" s="21" t="n">
-        <x:v>2.0818984029761385</x:v>
+        <x:v>0.8022035372906335</x:v>
       </x:c>
       <x:c r="J22" s="21" t="n">
-        <x:v>0.6099774136439187</x:v>
+        <x:v>0.5982537910095453</x:v>
       </x:c>
       <x:c r="K22" s="21" t="n">
-        <x:v>22.00767634600877</x:v>
+        <x:v>22.280339095724432</x:v>
       </x:c>
       <x:c r="L22" s="21" t="n">
-        <x:v>0.0005524728572880116</x:v>
+        <x:v>0.0012793929874142466</x:v>
       </x:c>
       <x:c r="M22" s="21" t="n">
-        <x:v>0.01872366710948112</x:v>
+        <x:v>0.04083359868834129</x:v>
       </x:c>
       <x:c r="N22" s="21" t="n">
+        <x:v>6.458333333333333</x:v>
+      </x:c>
+      <x:c r="O22" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1534,7 +1624,9 @@
       <x:c r="A23" t="str">
         <x:v>stage2_fine</x:v>
       </x:c>
-      <x:c r="B23" t="str"/>
+      <x:c r="B23" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C23" s="21" t="n">
         <x:v>0.025</x:v>
       </x:c>
@@ -1542,19 +1634,17 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E23" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F23" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G23" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="21" t="str"/>
+      <x:c r="G23" s="21" t="n">
+        <x:v>1.0524913310625879</x:v>
       </x:c>
       <x:c r="H23" s="21" t="n">
-        <x:v>0.7066252342175213</x:v>
+        <x:v>0.7097502342175211</x:v>
       </x:c>
       <x:c r="I23" s="21" t="n">
-        <x:v>0.9752444579327862</x:v>
+        <x:v>0.9773694579327863</x:v>
       </x:c>
       <x:c r="J23" s="21" t="n">
         <x:v>0.5969576006359417</x:v>
@@ -1569,18 +1659,21 @@
         <x:v>0.019451165080231727</x:v>
       </x:c>
       <x:c r="N23" s="21" t="n">
+        <x:v>3.125</x:v>
+      </x:c>
+      <x:c r="O23" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
-        <x:v>stage3_local</x:v>
+        <x:v>stage2_fine</x:v>
       </x:c>
       <x:c r="B24" t="n">
-        <x:v>1</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C24" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.075</x:v>
       </x:c>
       <x:c r="D24" s="21" t="n">
         <x:v>7</x:v>
@@ -1590,373 +1683,400 @@
       </x:c>
       <x:c r="F24" s="21" t="str"/>
       <x:c r="G24" s="21" t="n">
-        <x:v>1.5</x:v>
+        <x:v>1.2537933910753518</x:v>
       </x:c>
       <x:c r="H24" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8498769166154798</x:v>
       </x:c>
       <x:c r="I24" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>1.4250291152838965</x:v>
       </x:c>
       <x:c r="J24" s="21" t="n">
-        <x:v>0.7324137788938853</x:v>
+        <x:v>0.6873889356742513</x:v>
       </x:c>
       <x:c r="K24" s="21" t="n">
-        <x:v>34.517019466703736</x:v>
+        <x:v>28.767204004840345</x:v>
       </x:c>
       <x:c r="L24" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.00208202550290569</x:v>
       </x:c>
       <x:c r="M24" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>0.07495154535628075</x:v>
       </x:c>
       <x:c r="N24" s="21" t="n">
+        <x:v>11.982142857142856</x:v>
+      </x:c>
+      <x:c r="O24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B25" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B25" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C25" s="21" t="n">
-        <x:v>0.0005</x:v>
+        <x:v>0.06</x:v>
       </x:c>
       <x:c r="D25" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E25" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F25" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G25" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F25" s="21" t="str"/>
+      <x:c r="G25" s="21" t="n">
+        <x:v>1.33017072037316</x:v>
       </x:c>
       <x:c r="H25" s="21" t="n">
-        <x:v>1.0430373635009207</x:v>
+        <x:v>0.7461476419773082</x:v>
       </x:c>
       <x:c r="I25" s="21" t="n">
-        <x:v>1.1214517506927497</x:v>
+        <x:v>1.2675318913394567</x:v>
       </x:c>
       <x:c r="J25" s="21" t="n">
-        <x:v>0.7320670695632779</x:v>
+        <x:v>0.6158013818575379</x:v>
       </x:c>
       <x:c r="K25" s="21" t="n">
-        <x:v>33.79815261650994</x:v>
+        <x:v>23.572143130627598</x:v>
       </x:c>
       <x:c r="L25" s="21" t="n">
-        <x:v>0.00002293726800396141</x:v>
+        <x:v>0.0014257016895923564</x:v>
       </x:c>
       <x:c r="M25" s="21" t="n">
-        <x:v>0.001156126452759143</x:v>
+        <x:v>0.04764470316112936</x:v>
       </x:c>
       <x:c r="N25" s="21" t="n">
+        <x:v>7.553571428571429</x:v>
+      </x:c>
+      <x:c r="O25" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B26" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B26" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C26" s="21" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.0675</x:v>
       </x:c>
       <x:c r="D26" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E26" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F26" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G26" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="21" t="str"/>
+      <x:c r="G26" s="21" t="n">
+        <x:v>1.434746360190705</x:v>
       </x:c>
       <x:c r="H26" s="21" t="n">
-        <x:v>1.0346355769716085</x:v>
+        <x:v>0.8132798011143049</x:v>
       </x:c>
       <x:c r="I26" s="21" t="n">
-        <x:v>1.0962063171296366</x:v>
+        <x:v>1.3204485439899591</x:v>
       </x:c>
       <x:c r="J26" s="21" t="n">
-        <x:v>0.7300420300380823</x:v>
+        <x:v>0.6432172107121268</x:v>
       </x:c>
       <x:c r="K26" s="21" t="n">
-        <x:v>33.677008805443954</x:v>
+        <x:v>25.781432634376028</x:v>
       </x:c>
       <x:c r="L26" s="21" t="n">
-        <x:v>0.000047885167201105906</x:v>
+        <x:v>0.0017139838917762365</x:v>
       </x:c>
       <x:c r="M26" s="21" t="n">
-        <x:v>0.002292406554535129</x:v>
+        <x:v>0.05954732555229595</x:v>
       </x:c>
       <x:c r="N26" s="21" t="n">
+        <x:v>9.720238095238097</x:v>
+      </x:c>
+      <x:c r="O26" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B27" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B27" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C27" s="21" t="n">
-        <x:v>0.0015</x:v>
+        <x:v>0.0575</x:v>
       </x:c>
       <x:c r="D27" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E27" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F27" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G27" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="21" t="str"/>
+      <x:c r="G27" s="21" t="n">
+        <x:v>1.5633742254509144</x:v>
       </x:c>
       <x:c r="H27" s="21" t="n">
-        <x:v>1.0223997226975658</x:v>
+        <x:v>0.860214459944532</x:v>
       </x:c>
       <x:c r="I27" s="21" t="n">
-        <x:v>1.052109334755294</x:v>
+        <x:v>1.6066196973580462</x:v>
       </x:c>
       <x:c r="J27" s="21" t="n">
-        <x:v>0.7270169255457393</x:v>
+        <x:v>0.6140698818995249</x:v>
       </x:c>
       <x:c r="K27" s="21" t="n">
-        <x:v>33.759652901934665</x:v>
+        <x:v>23.373957468478483</x:v>
       </x:c>
       <x:c r="L27" s="21" t="n">
-        <x:v>0.00006992931591132707</x:v>
+        <x:v>0.0013892230997652048</x:v>
       </x:c>
       <x:c r="M27" s="21" t="n">
-        <x:v>0.0033199264582476724</x:v>
+        <x:v>0.04594636995698843</x:v>
       </x:c>
       <x:c r="N27" s="21" t="n">
+        <x:v>7.06547619047619</x:v>
+      </x:c>
+      <x:c r="O27" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B28" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B28" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C28" s="21" t="n">
-        <x:v>0.002</x:v>
+        <x:v>0.03</x:v>
       </x:c>
       <x:c r="D28" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E28" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F28" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G28" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F28" s="21" t="str"/>
+      <x:c r="G28" s="21" t="n">
+        <x:v>1.6053960666054639</x:v>
       </x:c>
       <x:c r="H28" s="21" t="n">
-        <x:v>1.0739415186707533</x:v>
+        <x:v>0.8687785837952972</x:v>
       </x:c>
       <x:c r="I28" s="21" t="n">
-        <x:v>1.178112094366953</x:v>
+        <x:v>1.5832754484701337</x:v>
       </x:c>
       <x:c r="J28" s="21" t="n">
-        <x:v>0.7258449760894597</x:v>
+        <x:v>0.58459134947737</x:v>
       </x:c>
       <x:c r="K28" s="21" t="n">
-        <x:v>33.504885038683135</x:v>
+        <x:v>20.63361888278891</x:v>
       </x:c>
       <x:c r="L28" s="21" t="n">
-        <x:v>0.00008450790190860864</x:v>
+        <x:v>0.000693100094956714</x:v>
       </x:c>
       <x:c r="M28" s="21" t="n">
-        <x:v>0.004053404167307004</x:v>
+        <x:v>0.021950022869046636</x:v>
       </x:c>
       <x:c r="N28" s="21" t="n">
+        <x:v>3.7857142857142856</x:v>
+      </x:c>
+      <x:c r="O28" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B29" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B29" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C29" s="21" t="n">
-        <x:v>0.0025</x:v>
+        <x:v>0.0725</x:v>
       </x:c>
       <x:c r="D29" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E29" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F29" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G29" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="21" t="str"/>
+      <x:c r="G29" s="21" t="n">
+        <x:v>1.6747960710032923</x:v>
       </x:c>
       <x:c r="H29" s="21" t="n">
-        <x:v>1.0270475665765908</x:v>
+        <x:v>0.9184618590969815</x:v>
       </x:c>
       <x:c r="I29" s="21" t="n">
-        <x:v>1.0666528404242814</x:v>
+        <x:v>1.5976322447070865</x:v>
       </x:c>
       <x:c r="J29" s="21" t="n">
-        <x:v>0.7215036643063957</x:v>
+        <x:v>0.6664276853075581</x:v>
       </x:c>
       <x:c r="K29" s="21" t="n">
-        <x:v>33.80561276626928</x:v>
+        <x:v>27.543603549727674</x:v>
       </x:c>
       <x:c r="L29" s="21" t="n">
-        <x:v>0.00009942141985853976</x:v>
+        <x:v>0.0018956230886195825</x:v>
       </x:c>
       <x:c r="M29" s="21" t="n">
-        <x:v>0.004861485797871268</x:v>
+        <x:v>0.06902999951054815</x:v>
       </x:c>
       <x:c r="N29" s="21" t="n">
+        <x:v>10.851190476190476</x:v>
+      </x:c>
+      <x:c r="O29" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B30" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C30" s="21" t="n">
-        <x:v>0.003</x:v>
+        <x:v>0.065</x:v>
       </x:c>
       <x:c r="D30" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E30" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F30" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G30" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" s="21" t="str"/>
+      <x:c r="G30" s="21" t="n">
+        <x:v>1.7075782854987447</x:v>
       </x:c>
       <x:c r="H30" s="21" t="n">
-        <x:v>0.9789043369389027</x:v>
+        <x:v>0.9195682450318458</x:v>
       </x:c>
       <x:c r="I30" s="21" t="n">
-        <x:v>1.0017774980497216</x:v>
+        <x:v>1.7267909300788005</x:v>
       </x:c>
       <x:c r="J30" s="21" t="n">
-        <x:v>0.7198791154127591</x:v>
+        <x:v>0.6353704263546566</x:v>
       </x:c>
       <x:c r="K30" s="21" t="n">
-        <x:v>33.71632231064082</x:v>
+        <x:v>24.873155679577625</x:v>
       </x:c>
       <x:c r="L30" s="21" t="n">
-        <x:v>0.0001174504784722918</x:v>
+        <x:v>0.0016404526597986874</x:v>
       </x:c>
       <x:c r="M30" s="21" t="n">
-        <x:v>0.005713171308973976</x:v>
+        <x:v>0.05474255298161521</x:v>
       </x:c>
       <x:c r="N30" s="21" t="n">
+        <x:v>8.767857142857142</x:v>
+      </x:c>
+      <x:c r="O30" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B31" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B31" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C31" s="21" t="n">
-        <x:v>0.0035</x:v>
+        <x:v>0.0275</x:v>
       </x:c>
       <x:c r="D31" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E31" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F31" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G31" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" s="21" t="str"/>
+      <x:c r="G31" s="21" t="n">
+        <x:v>1.8724181094079744</x:v>
       </x:c>
       <x:c r="H31" s="21" t="n">
-        <x:v>1.0216372788388572</x:v>
+        <x:v>0.9398287427771483</x:v>
       </x:c>
       <x:c r="I31" s="21" t="n">
-        <x:v>1.0624274699603415</x:v>
+        <x:v>2.260898485828972</x:v>
       </x:c>
       <x:c r="J31" s="21" t="n">
-        <x:v>0.7192461144561041</x:v>
+        <x:v>0.5864740104275107</x:v>
       </x:c>
       <x:c r="K31" s="21" t="n">
-        <x:v>33.24084411348541</x:v>
+        <x:v>20.797685421309694</x:v>
       </x:c>
       <x:c r="L31" s="21" t="n">
-        <x:v>0.00013589774416169562</x:v>
+        <x:v>0.0006333511806193362</x:v>
       </x:c>
       <x:c r="M31" s="21" t="n">
-        <x:v>0.00647285615856122</x:v>
+        <x:v>0.020496318171553916</x:v>
       </x:c>
       <x:c r="N31" s="21" t="n">
+        <x:v>3.5476190476190474</x:v>
+      </x:c>
+      <x:c r="O31" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
-        <x:v>stage3_local</x:v>
-      </x:c>
-      <x:c r="B32" t="str"/>
+        <x:v>stage2_fine</x:v>
+      </x:c>
+      <x:c r="B32" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C32" s="21" t="n">
-        <x:v>0.004</x:v>
+        <x:v>0.07</x:v>
       </x:c>
       <x:c r="D32" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E32" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F32" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G32" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" s="21" t="str"/>
+      <x:c r="G32" s="21" t="n">
+        <x:v>1.8988711250019332</x:v>
       </x:c>
       <x:c r="H32" s="21" t="n">
-        <x:v>1.0780047301799165</x:v>
+        <x:v>0.9926301536439588</x:v>
       </x:c>
       <x:c r="I32" s="21" t="n">
-        <x:v>1.176535445151257</x:v>
+        <x:v>2.0364893872427414</x:v>
       </x:c>
       <x:c r="J32" s="21" t="n">
-        <x:v>0.7172450760009489</x:v>
+        <x:v>0.6592519052625542</x:v>
       </x:c>
       <x:c r="K32" s="21" t="n">
-        <x:v>32.886495966380146</x:v>
+        <x:v>26.635902391049544</x:v>
       </x:c>
       <x:c r="L32" s="21" t="n">
-        <x:v>0.00015425917321751036</x:v>
+        <x:v>0.0018359761901217302</x:v>
       </x:c>
       <x:c r="M32" s="21" t="n">
-        <x:v>0.007258542648910503</x:v>
+        <x:v>0.06397448304853318</x:v>
       </x:c>
       <x:c r="N32" s="21" t="n">
+        <x:v>9.779761904761907</x:v>
+      </x:c>
+      <x:c r="O32" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>stage3_local</x:v>
+        <x:v>stage2_fine</x:v>
       </x:c>
       <x:c r="B33" t="str"/>
       <x:c r="C33" s="21" t="n">
-        <x:v>0.0045</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="D33" s="21" t="n">
         <x:v>7</x:v>
@@ -1965,30 +2085,33 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F33" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>premature_pause</x:v>
       </x:c>
       <x:c r="G33" s="21" t="str">
         <x:v>inf</x:v>
       </x:c>
       <x:c r="H33" s="21" t="n">
-        <x:v>1.066960361041747</x:v>
+        <x:v>0.9997806123881418</x:v>
       </x:c>
       <x:c r="I33" s="21" t="n">
-        <x:v>1.0896169405977374</x:v>
+        <x:v>1.7396761213378646</x:v>
       </x:c>
       <x:c r="J33" s="21" t="n">
-        <x:v>0.715465591249493</x:v>
+        <x:v>0.6263774702050323</x:v>
       </x:c>
       <x:c r="K33" s="21" t="n">
-        <x:v>32.94841897113552</x:v>
+        <x:v>24.124442070836363</x:v>
       </x:c>
       <x:c r="L33" s="21" t="n">
-        <x:v>0.00017268464879534315</x:v>
+        <x:v>0.0015502237230913716</x:v>
       </x:c>
       <x:c r="M33" s="21" t="n">
-        <x:v>0.008159268408167112</x:v>
+        <x:v>0.050918288533744624</x:v>
       </x:c>
       <x:c r="N33" s="21" t="n">
+        <x:v>7.8690476190476195</x:v>
+      </x:c>
+      <x:c r="O33" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1996,48 +2119,951 @@
       <x:c r="A34" t="str">
         <x:v>stage3_local</x:v>
       </x:c>
-      <x:c r="B34" t="str"/>
+      <x:c r="B34" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="C34" s="21" t="n">
-        <x:v>0.005</x:v>
+        <x:v>0.0415</x:v>
       </x:c>
       <x:c r="D34" s="21" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E34" s="22" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F34" s="21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
-      <x:c r="G34" s="21" t="str">
-        <x:v>inf</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" s="21" t="str"/>
+      <x:c r="G34" s="21" t="n">
+        <x:v>0.5858400877649983</x:v>
       </x:c>
       <x:c r="H34" s="21" t="n">
-        <x:v>1.0506585021333839</x:v>
+        <x:v>0.3994134205199783</x:v>
       </x:c>
       <x:c r="I34" s="21" t="n">
-        <x:v>1.0797285385370963</x:v>
+        <x:v>0.5853529172248085</x:v>
       </x:c>
       <x:c r="J34" s="21" t="n">
-        <x:v>0.7144184093790183</x:v>
+        <x:v>0.574999283796635</x:v>
       </x:c>
       <x:c r="K34" s="21" t="n">
-        <x:v>32.543069872365784</x:v>
+        <x:v>20.499985136541174</x:v>
       </x:c>
       <x:c r="L34" s="21" t="n">
-        <x:v>0.00018843105190779883</x:v>
+        <x:v>0.0009197803867279649</x:v>
       </x:c>
       <x:c r="M34" s="21" t="n">
-        <x:v>0.008829584942994512</x:v>
+        <x:v>0.02854773933939016</x:v>
       </x:c>
       <x:c r="N34" s="21" t="n">
+        <x:v>4.892857142857143</x:v>
+      </x:c>
+      <x:c r="O34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B35" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C35" s="21" t="n">
+        <x:v>0.0425</x:v>
+      </x:c>
+      <x:c r="D35" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E35" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="21" t="str"/>
+      <x:c r="G35" s="21" t="n">
+        <x:v>0.5879499406370574</x:v>
+      </x:c>
+      <x:c r="H35" s="21" t="n">
+        <x:v>0.4153507439082819</x:v>
+      </x:c>
+      <x:c r="I35" s="21" t="n">
+        <x:v>0.6329659406051644</x:v>
+      </x:c>
+      <x:c r="J35" s="21" t="n">
+        <x:v>0.5785728446559552</x:v>
+      </x:c>
+      <x:c r="K35" s="21" t="n">
+        <x:v>20.598195413255667</x:v>
+      </x:c>
+      <x:c r="L35" s="21" t="n">
+        <x:v>0.0009543818996144423</x:v>
+      </x:c>
+      <x:c r="M35" s="21" t="n">
+        <x:v>0.029398426514506637</x:v>
+      </x:c>
+      <x:c r="N35" s="21" t="n">
+        <x:v>4.845238095238096</x:v>
+      </x:c>
+      <x:c r="O35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B36" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C36" s="21" t="n">
+        <x:v>0.0405</x:v>
+      </x:c>
+      <x:c r="D36" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E36" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F36" s="21" t="str"/>
+      <x:c r="G36" s="21" t="n">
+        <x:v>0.6127062652924536</x:v>
+      </x:c>
+      <x:c r="H36" s="21" t="n">
+        <x:v>0.4138498927851453</x:v>
+      </x:c>
+      <x:c r="I36" s="21" t="n">
+        <x:v>0.5547146145519082</x:v>
+      </x:c>
+      <x:c r="J36" s="21" t="n">
+        <x:v>0.5733911441791305</x:v>
+      </x:c>
+      <x:c r="K36" s="21" t="n">
+        <x:v>20.414584241108077</x:v>
+      </x:c>
+      <x:c r="L36" s="21" t="n">
+        <x:v>0.0008952735327337201</x:v>
+      </x:c>
+      <x:c r="M36" s="21" t="n">
+        <x:v>0.02780930478606119</x:v>
+      </x:c>
+      <x:c r="N36" s="21" t="n">
+        <x:v>4.755952380952381</x:v>
+      </x:c>
+      <x:c r="O36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B37" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C37" s="21" t="n">
+        <x:v>0.0475</x:v>
+      </x:c>
+      <x:c r="D37" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E37" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F37" s="21" t="str"/>
+      <x:c r="G37" s="21" t="n">
+        <x:v>0.6231404368575117</x:v>
+      </x:c>
+      <x:c r="H37" s="21" t="n">
+        <x:v>0.3903972793717462</x:v>
+      </x:c>
+      <x:c r="I37" s="21" t="n">
+        <x:v>0.7833822924878484</x:v>
+      </x:c>
+      <x:c r="J37" s="21" t="n">
+        <x:v>0.5848557285559549</x:v>
+      </x:c>
+      <x:c r="K37" s="21" t="n">
+        <x:v>21.173191272766253</x:v>
+      </x:c>
+      <x:c r="L37" s="21" t="n">
+        <x:v>0.0010615376969566204</x:v>
+      </x:c>
+      <x:c r="M37" s="21" t="n">
+        <x:v>0.03348034548688624</x:v>
+      </x:c>
+      <x:c r="N37" s="21" t="n">
+        <x:v>5.136904761904762</x:v>
+      </x:c>
+      <x:c r="O37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B38" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C38" s="21" t="n">
+        <x:v>0.0435</x:v>
+      </x:c>
+      <x:c r="D38" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E38" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F38" s="21" t="str"/>
+      <x:c r="G38" s="21" t="n">
+        <x:v>0.6446143562170031</x:v>
+      </x:c>
+      <x:c r="H38" s="21" t="n">
+        <x:v>0.4422480104208966</x:v>
+      </x:c>
+      <x:c r="I38" s="21" t="n">
+        <x:v>0.677370760939178</x:v>
+      </x:c>
+      <x:c r="J38" s="21" t="n">
+        <x:v>0.5793521138332469</x:v>
+      </x:c>
+      <x:c r="K38" s="21" t="n">
+        <x:v>20.544024768452594</x:v>
+      </x:c>
+      <x:c r="L38" s="21" t="n">
+        <x:v>0.0009814632011650845</x:v>
+      </x:c>
+      <x:c r="M38" s="21" t="n">
+        <x:v>0.02983172044543969</x:v>
+      </x:c>
+      <x:c r="N38" s="21" t="n">
+        <x:v>4.732142857142857</x:v>
+      </x:c>
+      <x:c r="O38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B39" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C39" s="21" t="n">
+        <x:v>0.045</x:v>
+      </x:c>
+      <x:c r="D39" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E39" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F39" s="21" t="str"/>
+      <x:c r="G39" s="21" t="n">
+        <x:v>0.6688585407275436</x:v>
+      </x:c>
+      <x:c r="H39" s="21" t="n">
+        <x:v>0.4609825115381697</x:v>
+      </x:c>
+      <x:c r="I39" s="21" t="n">
+        <x:v>0.5469503295641454</x:v>
+      </x:c>
+      <x:c r="J39" s="21" t="n">
+        <x:v>0.5829696426603963</x:v>
+      </x:c>
+      <x:c r="K39" s="21" t="n">
+        <x:v>20.671351753002295</x:v>
+      </x:c>
+      <x:c r="L39" s="21" t="n">
+        <x:v>0.0010099097878908904</x:v>
+      </x:c>
+      <x:c r="M39" s="21" t="n">
+        <x:v>0.030771802061914478</x:v>
+      </x:c>
+      <x:c r="N39" s="21" t="n">
+        <x:v>4.916666666666666</x:v>
+      </x:c>
+      <x:c r="O39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B40" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C40" s="21" t="n">
+        <x:v>0.044</x:v>
+      </x:c>
+      <x:c r="D40" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E40" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F40" s="21" t="str"/>
+      <x:c r="G40" s="21" t="n">
+        <x:v>0.6703156206767755</x:v>
+      </x:c>
+      <x:c r="H40" s="21" t="n">
+        <x:v>0.446474944736035</x:v>
+      </x:c>
+      <x:c r="I40" s="21" t="n">
+        <x:v>0.49944204118757884</x:v>
+      </x:c>
+      <x:c r="J40" s="21" t="n">
+        <x:v>0.5823405185390138</x:v>
+      </x:c>
+      <x:c r="K40" s="21" t="n">
+        <x:v>20.63618154505024</x:v>
+      </x:c>
+      <x:c r="L40" s="21" t="n">
+        <x:v>0.0009956655963390465</x:v>
+      </x:c>
+      <x:c r="M40" s="21" t="n">
+        <x:v>0.0303181465227487</x:v>
+      </x:c>
+      <x:c r="N40" s="21" t="n">
+        <x:v>4.863095238095238</x:v>
+      </x:c>
+      <x:c r="O40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C41" s="21" t="n">
+        <x:v>0.039</x:v>
+      </x:c>
+      <x:c r="D41" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E41" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F41" s="21" t="str"/>
+      <x:c r="G41" s="21" t="n">
+        <x:v>0.7008608053782015</x:v>
+      </x:c>
+      <x:c r="H41" s="21" t="n">
+        <x:v>0.4573781672955616</x:v>
+      </x:c>
+      <x:c r="I41" s="21" t="n">
+        <x:v>0.5848813225992601</x:v>
+      </x:c>
+      <x:c r="J41" s="21" t="n">
+        <x:v>0.5748866344285414</x:v>
+      </x:c>
+      <x:c r="K41" s="21" t="n">
+        <x:v>20.364783950361094</x:v>
+      </x:c>
+      <x:c r="L41" s="21" t="n">
+        <x:v>0.0008650186619533935</x:v>
+      </x:c>
+      <x:c r="M41" s="21" t="n">
+        <x:v>0.026786374606365255</x:v>
+      </x:c>
+      <x:c r="N41" s="21" t="n">
+        <x:v>4.577380952380953</x:v>
+      </x:c>
+      <x:c r="O41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B42" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C42" s="21" t="n">
+        <x:v>0.0445</x:v>
+      </x:c>
+      <x:c r="D42" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E42" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F42" s="21" t="str"/>
+      <x:c r="G42" s="21" t="n">
+        <x:v>0.7717459212760709</x:v>
+      </x:c>
+      <x:c r="H42" s="21" t="n">
+        <x:v>0.5022766651863543</x:v>
+      </x:c>
+      <x:c r="I42" s="21" t="n">
+        <x:v>0.7182606279790632</x:v>
+      </x:c>
+      <x:c r="J42" s="21" t="n">
+        <x:v>0.5808046122766436</x:v>
+      </x:c>
+      <x:c r="K42" s="21" t="n">
+        <x:v>20.61643764666163</x:v>
+      </x:c>
+      <x:c r="L42" s="21" t="n">
+        <x:v>0.0010048204119096934</x:v>
+      </x:c>
+      <x:c r="M42" s="21" t="n">
+        <x:v>0.030482718865918763</x:v>
+      </x:c>
+      <x:c r="N42" s="21" t="n">
+        <x:v>4.875</x:v>
+      </x:c>
+      <x:c r="O42" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B43" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C43" s="21" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="D43" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E43" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F43" s="21" t="str"/>
+      <x:c r="G43" s="21" t="n">
+        <x:v>0.8313096468709749</x:v>
+      </x:c>
+      <x:c r="H43" s="21" t="n">
+        <x:v>0.5462156895750908</x:v>
+      </x:c>
+      <x:c r="I43" s="21" t="n">
+        <x:v>0.9412516624258085</x:v>
+      </x:c>
+      <x:c r="J43" s="21" t="n">
+        <x:v>0.5782834299435242</x:v>
+      </x:c>
+      <x:c r="K43" s="21" t="n">
+        <x:v>20.33680183680493</x:v>
+      </x:c>
+      <x:c r="L43" s="21" t="n">
+        <x:v>0.0009063263727419075</x:v>
+      </x:c>
+      <x:c r="M43" s="21" t="n">
+        <x:v>0.027300113650715264</x:v>
+      </x:c>
+      <x:c r="N43" s="21" t="n">
+        <x:v>4.553571428571429</x:v>
+      </x:c>
+      <x:c r="O43" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B44" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C44" s="21" t="n">
+        <x:v>0.0465</x:v>
+      </x:c>
+      <x:c r="D44" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E44" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F44" s="21" t="str"/>
+      <x:c r="G44" s="21" t="n">
+        <x:v>0.8358381670067518</x:v>
+      </x:c>
+      <x:c r="H44" s="21" t="n">
+        <x:v>0.5624587049874537</x:v>
+      </x:c>
+      <x:c r="I44" s="21" t="n">
+        <x:v>0.7664951043885639</x:v>
+      </x:c>
+      <x:c r="J44" s="21" t="n">
+        <x:v>0.589374367801606</x:v>
+      </x:c>
+      <x:c r="K44" s="21" t="n">
+        <x:v>20.98889180197899</x:v>
+      </x:c>
+      <x:c r="L44" s="21" t="n">
+        <x:v>0.0010690494780596323</x:v>
+      </x:c>
+      <x:c r="M44" s="21" t="n">
+        <x:v>0.03254829761325803</x:v>
+      </x:c>
+      <x:c r="N44" s="21" t="n">
+        <x:v>5.0178571428571415</x:v>
+      </x:c>
+      <x:c r="O44" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B45" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C45" s="21" t="n">
+        <x:v>0.041</x:v>
+      </x:c>
+      <x:c r="D45" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E45" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F45" s="21" t="str"/>
+      <x:c r="G45" s="21" t="n">
+        <x:v>0.9312399109081485</x:v>
+      </x:c>
+      <x:c r="H45" s="21" t="n">
+        <x:v>0.5667350154760606</x:v>
+      </x:c>
+      <x:c r="I45" s="21" t="n">
+        <x:v>0.8587387293624401</x:v>
+      </x:c>
+      <x:c r="J45" s="21" t="n">
+        <x:v>0.5774392314261473</x:v>
+      </x:c>
+      <x:c r="K45" s="21" t="n">
+        <x:v>20.46285225768139</x:v>
+      </x:c>
+      <x:c r="L45" s="21" t="n">
+        <x:v>0.000927350374024822</x:v>
+      </x:c>
+      <x:c r="M45" s="21" t="n">
+        <x:v>0.028250400821643935</x:v>
+      </x:c>
+      <x:c r="N45" s="21" t="n">
+        <x:v>4.690476190476191</x:v>
+      </x:c>
+      <x:c r="O45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B46" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C46" s="21" t="n">
+        <x:v>0.043</x:v>
+      </x:c>
+      <x:c r="D46" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E46" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F46" s="21" t="str"/>
+      <x:c r="G46" s="21" t="n">
+        <x:v>0.9324308463730193</x:v>
+      </x:c>
+      <x:c r="H46" s="21" t="n">
+        <x:v>0.5445858072511639</x:v>
+      </x:c>
+      <x:c r="I46" s="21" t="n">
+        <x:v>0.7982382758563115</x:v>
+      </x:c>
+      <x:c r="J46" s="21" t="n">
+        <x:v>0.5873673558101359</x:v>
+      </x:c>
+      <x:c r="K46" s="21" t="n">
+        <x:v>20.583970528427255</x:v>
+      </x:c>
+      <x:c r="L46" s="21" t="n">
+        <x:v>0.0009904295593108827</x:v>
+      </x:c>
+      <x:c r="M46" s="21" t="n">
+        <x:v>0.029675421288410695</x:v>
+      </x:c>
+      <x:c r="N46" s="21" t="n">
+        <x:v>4.821428571428571</x:v>
+      </x:c>
+      <x:c r="O46" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B47" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C47" s="21" t="n">
+        <x:v>0.0455</x:v>
+      </x:c>
+      <x:c r="D47" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E47" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F47" s="21" t="str"/>
+      <x:c r="G47" s="21" t="n">
+        <x:v>0.9388837487671444</x:v>
+      </x:c>
+      <x:c r="H47" s="21" t="n">
+        <x:v>0.6180508204520725</x:v>
+      </x:c>
+      <x:c r="I47" s="21" t="n">
+        <x:v>0.754440922389699</x:v>
+      </x:c>
+      <x:c r="J47" s="21" t="n">
+        <x:v>0.5924697337629503</x:v>
+      </x:c>
+      <x:c r="K47" s="21" t="n">
+        <x:v>20.723034820736164</x:v>
+      </x:c>
+      <x:c r="L47" s="21" t="n">
+        <x:v>0.0010501039314168741</x:v>
+      </x:c>
+      <x:c r="M47" s="21" t="n">
+        <x:v>0.03111930378650691</x:v>
+      </x:c>
+      <x:c r="N47" s="21" t="n">
+        <x:v>5.136904761904762</x:v>
+      </x:c>
+      <x:c r="O47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B48" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C48" s="21" t="n">
+        <x:v>0.0395</x:v>
+      </x:c>
+      <x:c r="D48" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E48" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F48" s="21" t="str"/>
+      <x:c r="G48" s="21" t="n">
+        <x:v>0.9499992507473393</x:v>
+      </x:c>
+      <x:c r="H48" s="21" t="n">
+        <x:v>0.5853325213268423</x:v>
+      </x:c>
+      <x:c r="I48" s="21" t="n">
+        <x:v>0.8790944154160646</x:v>
+      </x:c>
+      <x:c r="J48" s="21" t="n">
+        <x:v>0.578571430444249</x:v>
+      </x:c>
+      <x:c r="K48" s="21" t="n">
+        <x:v>20.40939105277104</x:v>
+      </x:c>
+      <x:c r="L48" s="21" t="n">
+        <x:v>0.0008945845692314124</x:v>
+      </x:c>
+      <x:c r="M48" s="21" t="n">
+        <x:v>0.02721957753800569</x:v>
+      </x:c>
+      <x:c r="N48" s="21" t="n">
+        <x:v>4.440476190476191</x:v>
+      </x:c>
+      <x:c r="O48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B49" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C49" s="21" t="n">
+        <x:v>0.042</x:v>
+      </x:c>
+      <x:c r="D49" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E49" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F49" s="21" t="str"/>
+      <x:c r="G49" s="21" t="n">
+        <x:v>0.9685280679664254</x:v>
+      </x:c>
+      <x:c r="H49" s="21" t="n">
+        <x:v>0.5889613450073845</x:v>
+      </x:c>
+      <x:c r="I49" s="21" t="n">
+        <x:v>0.8808724708161368</x:v>
+      </x:c>
+      <x:c r="J49" s="21" t="n">
+        <x:v>0.5792213324566414</x:v>
+      </x:c>
+      <x:c r="K49" s="21" t="n">
+        <x:v>20.525309188801405</x:v>
+      </x:c>
+      <x:c r="L49" s="21" t="n">
+        <x:v>0.0009511866495355706</x:v>
+      </x:c>
+      <x:c r="M49" s="21" t="n">
+        <x:v>0.028882934113066642</x:v>
+      </x:c>
+      <x:c r="N49" s="21" t="n">
+        <x:v>4.898809523809524</x:v>
+      </x:c>
+      <x:c r="O49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B50" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C50" s="21" t="n">
+        <x:v>0.0375</x:v>
+      </x:c>
+      <x:c r="D50" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E50" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F50" s="21" t="str"/>
+      <x:c r="G50" s="21" t="n">
+        <x:v>0.990114187197696</x:v>
+      </x:c>
+      <x:c r="H50" s="21" t="n">
+        <x:v>0.634110600555118</x:v>
+      </x:c>
+      <x:c r="I50" s="21" t="n">
+        <x:v>0.9084012417761826</x:v>
+      </x:c>
+      <x:c r="J50" s="21" t="n">
+        <x:v>0.5820238621281989</x:v>
+      </x:c>
+      <x:c r="K50" s="21" t="n">
+        <x:v>20.308352579412112</x:v>
+      </x:c>
+      <x:c r="L50" s="21" t="n">
+        <x:v>0.0008576574770892432</x:v>
+      </x:c>
+      <x:c r="M50" s="21" t="n">
+        <x:v>0.02579059223383672</x:v>
+      </x:c>
+      <x:c r="N50" s="21" t="n">
+        <x:v>4.035714285714286</x:v>
+      </x:c>
+      <x:c r="O50" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B51" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C51" s="21" t="n">
+        <x:v>0.0385</x:v>
+      </x:c>
+      <x:c r="D51" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E51" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F51" s="21" t="str"/>
+      <x:c r="G51" s="21" t="n">
+        <x:v>1.108382871834267</x:v>
+      </x:c>
+      <x:c r="H51" s="21" t="n">
+        <x:v>0.6738495355632559</x:v>
+      </x:c>
+      <x:c r="I51" s="21" t="n">
+        <x:v>0.892496197075593</x:v>
+      </x:c>
+      <x:c r="J51" s="21" t="n">
+        <x:v>0.5824742919925044</x:v>
+      </x:c>
+      <x:c r="K51" s="21" t="n">
+        <x:v>20.385555278941986</x:v>
+      </x:c>
+      <x:c r="L51" s="21" t="n">
+        <x:v>0.0008851410201995454</x:v>
+      </x:c>
+      <x:c r="M51" s="21" t="n">
+        <x:v>0.02661532428824465</x:v>
+      </x:c>
+      <x:c r="N51" s="21" t="n">
+        <x:v>4.3273809523809526</x:v>
+      </x:c>
+      <x:c r="O51" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B52" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C52" s="21" t="n">
+        <x:v>0.046</x:v>
+      </x:c>
+      <x:c r="D52" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E52" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F52" s="21" t="str"/>
+      <x:c r="G52" s="21" t="n">
+        <x:v>1.1344692419093212</x:v>
+      </x:c>
+      <x:c r="H52" s="21" t="n">
+        <x:v>0.6214502102821545</x:v>
+      </x:c>
+      <x:c r="I52" s="21" t="n">
+        <x:v>0.9869642665542562</x:v>
+      </x:c>
+      <x:c r="J52" s="21" t="n">
+        <x:v>0.5833230600848479</x:v>
+      </x:c>
+      <x:c r="K52" s="21" t="n">
+        <x:v>20.92681261880616</x:v>
+      </x:c>
+      <x:c r="L52" s="21" t="n">
+        <x:v>0.0010335867589965186</x:v>
+      </x:c>
+      <x:c r="M52" s="21" t="n">
+        <x:v>0.03203491554581686</x:v>
+      </x:c>
+      <x:c r="N52" s="21" t="n">
+        <x:v>5.017857142857143</x:v>
+      </x:c>
+      <x:c r="O52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B53" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C53" s="21" t="n">
+        <x:v>0.047</x:v>
+      </x:c>
+      <x:c r="D53" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E53" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F53" s="21" t="str"/>
+      <x:c r="G53" s="21" t="n">
+        <x:v>1.1943412111126936</x:v>
+      </x:c>
+      <x:c r="H53" s="21" t="n">
+        <x:v>0.6552717528475885</x:v>
+      </x:c>
+      <x:c r="I53" s="21" t="n">
+        <x:v>1.052081435862797</x:v>
+      </x:c>
+      <x:c r="J53" s="21" t="n">
+        <x:v>0.5852311299414504</x:v>
+      </x:c>
+      <x:c r="K53" s="21" t="n">
+        <x:v>21.007800132188088</x:v>
+      </x:c>
+      <x:c r="L53" s="21" t="n">
+        <x:v>0.0010570596835107239</x:v>
+      </x:c>
+      <x:c r="M53" s="21" t="n">
+        <x:v>0.03273733127135597</x:v>
+      </x:c>
+      <x:c r="N53" s="21" t="n">
+        <x:v>5.1607142857142865</x:v>
+      </x:c>
+      <x:c r="O53" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>stage3_local</x:v>
+      </x:c>
+      <x:c r="B54" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C54" s="21" t="n">
+        <x:v>0.038</x:v>
+      </x:c>
+      <x:c r="D54" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E54" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F54" s="21" t="str"/>
+      <x:c r="G54" s="21" t="n">
+        <x:v>1.5771066292884133</x:v>
+      </x:c>
+      <x:c r="H54" s="21" t="n">
+        <x:v>0.8789360778267287</x:v>
+      </x:c>
+      <x:c r="I54" s="21" t="n">
+        <x:v>1.2567336441288568</x:v>
+      </x:c>
+      <x:c r="J54" s="21" t="n">
+        <x:v>0.5836287229521762</x:v>
+      </x:c>
+      <x:c r="K54" s="21" t="n">
+        <x:v>20.274789496037126</x:v>
+      </x:c>
+      <x:c r="L54" s="21" t="n">
+        <x:v>0.0008883247009560453</x:v>
+      </x:c>
+      <x:c r="M54" s="21" t="n">
+        <x:v>0.02602902494925822</x:v>
+      </x:c>
+      <x:c r="N54" s="21" t="n">
+        <x:v>4.166666666666666</x:v>
+      </x:c>
+      <x:c r="O54" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3deca6dff8c4e98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4866bf3b43fb446e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2060,7 +3086,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>Old PR #20 reference is shown for comparison only; it is hard-rejected under the merged Pitch controller because it saturates the simulation-only Moving-mass actuator.</x:v>
+        <x:v>Old PR #20 reference is shown for comparison only; it is hard-rejected under the merged Pitch controller for excessive Moving-mass rate/acceleration limiter duty and duration.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2077,7 +3103,7 @@
         <x:v>Selected</x:v>
       </x:c>
       <x:c r="E3" s="10" t="str">
-        <x:v>Selected vs gain 0</x:v>
+        <x:v>Selected minus gain 0</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2091,10 +3117,10 @@
         <x:v>1.0856988477598764</x:v>
       </x:c>
       <x:c r="D4" s="12" t="n">
-        <x:v>0.5255464177915979</x:v>
-      </x:c>
-      <x:c r="E4" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.05369817951286041</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="n">
+        <x:v>-0.4718482382787375</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2108,10 +3134,10 @@
         <x:v>10.490676146122007</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
-        <x:v>2.37222359161449</x:v>
-      </x:c>
-      <x:c r="E5" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0296304817888938</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="n">
+        <x:v>-2.342593109825596</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2125,10 +3151,10 @@
         <x:v>0.039889226064712506</x:v>
       </x:c>
       <x:c r="D6" s="12" t="n">
-        <x:v>0.03023908845187382</x:v>
-      </x:c>
-      <x:c r="E6" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.015021716924069747</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="n">
+        <x:v>-0.015217371527804073</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2142,10 +3168,10 @@
         <x:v>0.08468901268379135</x:v>
       </x:c>
       <x:c r="D7" s="12" t="n">
-        <x:v>0.06313959546321832</x:v>
-      </x:c>
-      <x:c r="E7" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.03395765511375735</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="n">
+        <x:v>-0.02918194034946097</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2159,10 +3185,10 @@
         <x:v>0.011098083835853806</x:v>
       </x:c>
       <x:c r="D8" s="12" t="n">
-        <x:v>0.01736159035498888</x:v>
-      </x:c>
-      <x:c r="E8" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.022014443742606724</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="n">
+        <x:v>0.0046528533876178425</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2176,10 +3202,10 @@
         <x:v>0.33103831359277625</x:v>
       </x:c>
       <x:c r="D9" s="12" t="n">
-        <x:v>0.3301493683863709</x:v>
-      </x:c>
-      <x:c r="E9" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.33792262344342333</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="n">
+        <x:v>0.007773255057052453</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2193,10 +3219,10 @@
         <x:v>0.5893382924613062</x:v>
       </x:c>
       <x:c r="D10" s="12" t="n">
-        <x:v>0.5851838806518579</x:v>
-      </x:c>
-      <x:c r="E10" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.5833862580133234</x:v>
+      </x:c>
+      <x:c r="E10" s="12" t="n">
+        <x:v>-0.0017976226385344463</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2210,10 +3236,10 @@
         <x:v>9.692142857143088</x:v>
       </x:c>
       <x:c r="D11" s="12" t="n">
-        <x:v>5.134285714285655</x:v>
-      </x:c>
-      <x:c r="E11" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>5.129999999999946</x:v>
+      </x:c>
+      <x:c r="E11" s="12" t="n">
+        <x:v>-0.004285714285709119</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2227,10 +3253,10 @@
         <x:v>1.8244210288332037</x:v>
       </x:c>
       <x:c r="D12" s="12" t="n">
-        <x:v>0.7324137788938853</x:v>
-      </x:c>
-      <x:c r="E12" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.574999283796635</x:v>
+      </x:c>
+      <x:c r="E12" s="12" t="n">
+        <x:v>-0.15741449509725025</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2244,10 +3270,10 @@
         <x:v>170.13051968890676</x:v>
       </x:c>
       <x:c r="D13" s="12" t="n">
-        <x:v>34.517019466703736</x:v>
-      </x:c>
-      <x:c r="E13" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>20.499985136541174</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="n">
+        <x:v>-14.017034330162563</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2261,10 +3287,10 @@
         <x:v>40.17700356065404</x:v>
       </x:c>
       <x:c r="D14" s="12" t="n">
-        <x:v>30.716419702006515</x:v>
-      </x:c>
-      <x:c r="E14" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>30.757650711958565</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="n">
+        <x:v>0.041231009952049646</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2278,10 +3304,10 @@
         <x:v>0.008011023623836698</x:v>
       </x:c>
       <x:c r="D15" s="12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E15" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0009197803867279649</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="n">
+        <x:v>0.0009197803867279649</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2295,10 +3321,10 @@
         <x:v>0.6996131934251938</x:v>
       </x:c>
       <x:c r="D16" s="12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E16" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.02854773933939016</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="n">
+        <x:v>0.02854773933939016</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2312,10 +3338,10 @@
         <x:v>0.07876968503121659</x:v>
       </x:c>
       <x:c r="D17" s="12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.011025898630469513</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="n">
+        <x:v>0.011025898630469513</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2329,10 +3355,129 @@
         <x:v>0.8895957941012086</x:v>
       </x:c>
       <x:c r="D18" s="12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.29810266938515995</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="n">
+        <x:v>0.29810266938515995</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>moving_mass_max_abs_offset_m</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="n">
+        <x:v>0.014159948849705879</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="n">
+        <x:v>0.006535912860134378</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="n">
+        <x:v>0.006535912860134378</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>moving_mass_max_abs_velocity_m_s</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="n">
+        <x:v>0.15899099518441226</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="n">
+        <x:v>0.09341387912770648</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="n">
+        <x:v>0.09341387912770648</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>moving_mass_max_abs_acceleration_m_s2</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="n">
+        <x:v>1.000000000000022</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="n">
+        <x:v>1.000000000000022</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>moving_mass_command_clipping_duty_percent</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C22" s="12" t="n">
+        <x:v>0.21428571428571427</x:v>
+      </x:c>
+      <x:c r="D22" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>moving_mass_rail_contact_duty_percent</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C23" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>moving_mass_rate_limiter_duty_percent</x:v>
+      </x:c>
+      <x:c r="B24" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C24" s="12" t="n">
+        <x:v>51.06547619047619</x:v>
+      </x:c>
+      <x:c r="D24" s="12" t="n">
+        <x:v>0.17857142857142858</x:v>
+      </x:c>
+      <x:c r="E24" s="12" t="n">
+        <x:v>0.17857142857142858</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>moving_mass_acceleration_limiter_duty_percent</x:v>
+      </x:c>
+      <x:c r="B25" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C25" s="12" t="n">
+        <x:v>82.23214285714286</x:v>
+      </x:c>
+      <x:c r="D25" s="12" t="n">
+        <x:v>4.892857142857143</x:v>
+      </x:c>
+      <x:c r="E25" s="12" t="n">
+        <x:v>4.892857142857143</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2342,7 +3487,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6b29fde6fd0403a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce24b851ab8f4183"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2499,7 +3644,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="E3" s="20" t="b">
         <x:v>0</x:v>
@@ -2586,10 +3731,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N4" t="n">
-        <x:v>0</x:v>
+        <x:v>5.541666666666667</x:v>
       </x:c>
       <x:c r="O4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P4" t="n">
         <x:v>0</x:v>
@@ -2672,7 +3817,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="E6" s="20" t="b">
         <x:v>0</x:v>
@@ -2759,10 +3904,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N7" t="n">
-        <x:v>0</x:v>
+        <x:v>5.541666666666667</x:v>
       </x:c>
       <x:c r="O7" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P7" t="n">
         <x:v>0</x:v>
@@ -2845,7 +3990,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="E9" s="20" t="b">
         <x:v>0</x:v>
@@ -2932,7 +4077,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N10" t="n">
-        <x:v>0</x:v>
+        <x:v>4.291666666666667</x:v>
       </x:c>
       <x:c r="O10" t="n">
         <x:v>1</x:v>
@@ -3018,7 +4163,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="E12" s="20" t="b">
         <x:v>0</x:v>
@@ -3105,7 +4250,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N13" t="n">
-        <x:v>0</x:v>
+        <x:v>4.291666666666667</x:v>
       </x:c>
       <x:c r="O13" t="n">
         <x:v>1</x:v>
@@ -3191,7 +4336,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="E15" s="20" t="b">
         <x:v>0</x:v>
@@ -3278,10 +4423,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N16" t="n">
-        <x:v>0</x:v>
+        <x:v>5.75</x:v>
       </x:c>
       <x:c r="O16" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P16" t="n">
         <x:v>0</x:v>
@@ -3364,7 +4509,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="E18" s="20" t="b">
         <x:v>0</x:v>
@@ -3451,10 +4596,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N19" t="n">
-        <x:v>0</x:v>
+        <x:v>5.75</x:v>
       </x:c>
       <x:c r="O19" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P19" t="n">
         <x:v>0</x:v>
@@ -3534,11 +4679,9 @@
         <x:v>old_pr20_reference_0_1325</x:v>
       </x:c>
       <x:c r="C21" s="20" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D21" t="str">
-        <x:v>moving_mass_saturation; moving_mass_acceleration_limit</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" t="str"/>
       <x:c r="E21" s="20" t="b">
         <x:v>0</x:v>
       </x:c>
@@ -3624,10 +4767,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N22" t="n">
-        <x:v>0</x:v>
+        <x:v>3.0833333333333335</x:v>
       </x:c>
       <x:c r="O22" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P22" t="n">
         <x:v>0</x:v>
@@ -3645,12 +4788,1059 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R503456be21cb46e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46afc51e2124966"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Moving-mass Limiter Duty, Duration, and Actual Maxima</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="18" t="str">
+        <x:v>Hard gates: command clipping/rail contact &gt;5% or &gt;0.5 s; rate limiting &gt;20% or &gt;1.0 s; acceleration limiting &gt;30% or &gt;1.0 s. Actual offset/rate/acceleration violations use max + 1e-9.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="10" t="str">
+        <x:v>Scenario</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>Controller set</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="str">
+        <x:v>Command clip duty %</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>Command clip longest s</x:v>
+      </x:c>
+      <x:c r="F3" s="10" t="str">
+        <x:v>Rail contact duty %</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str">
+        <x:v>Rail contact longest s</x:v>
+      </x:c>
+      <x:c r="H3" s="10" t="str">
+        <x:v>Rate limiter duty %</x:v>
+      </x:c>
+      <x:c r="I3" s="10" t="str">
+        <x:v>Rate limiter longest s</x:v>
+      </x:c>
+      <x:c r="J3" s="10" t="str">
+        <x:v>Accel limiter duty %</x:v>
+      </x:c>
+      <x:c r="K3" s="10" t="str">
+        <x:v>Accel limiter longest s</x:v>
+      </x:c>
+      <x:c r="L3" s="10" t="str">
+        <x:v>Actual max offset m</x:v>
+      </x:c>
+      <x:c r="M3" s="10" t="str">
+        <x:v>Actual max rate m/s</x:v>
+      </x:c>
+      <x:c r="N3" s="10" t="str">
+        <x:v>Actual max accel m/s²</x:v>
+      </x:c>
+      <x:c r="O3" s="10" t="str">
+        <x:v>Reasons</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>loiter_positive_disturbance</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>gain_zero_baseline</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>loiter_positive_disturbance</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>old_pr20_reference_0_1325</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="21" t="n">
+        <x:v>57.75</x:v>
+      </x:c>
+      <x:c r="I5" s="21" t="n">
+        <x:v>0.25999999999999446</x:v>
+      </x:c>
+      <x:c r="J5" s="21" t="n">
+        <x:v>90.5</x:v>
+      </x:c>
+      <x:c r="K5" s="21" t="n">
+        <x:v>2.2299999999999525</x:v>
+      </x:c>
+      <x:c r="L5" s="21" t="n">
+        <x:v>0.016717546900312342</x:v>
+      </x:c>
+      <x:c r="M5" s="21" t="n">
+        <x:v>0.17344054841769865</x:v>
+      </x:c>
+      <x:c r="N5" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>loiter_positive_disturbance</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>selected</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="21" t="n">
+        <x:v>5.541666666666667</x:v>
+      </x:c>
+      <x:c r="K6" s="21" t="n">
+        <x:v>0.42999999999999083</x:v>
+      </x:c>
+      <x:c r="L6" s="21" t="n">
+        <x:v>0.00864535302490578</x:v>
+      </x:c>
+      <x:c r="M6" s="21" t="n">
+        <x:v>0.12198570161509474</x:v>
+      </x:c>
+      <x:c r="N6" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>loiter_negative_disturbance</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>gain_zero_baseline</x:v>
+      </x:c>
+      <x:c r="C7" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N7" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>loiter_negative_disturbance</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>old_pr20_reference_0_1325</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="21" t="n">
+        <x:v>57.75</x:v>
+      </x:c>
+      <x:c r="I8" s="21" t="n">
+        <x:v>0.25999999999999446</x:v>
+      </x:c>
+      <x:c r="J8" s="21" t="n">
+        <x:v>90.5</x:v>
+      </x:c>
+      <x:c r="K8" s="21" t="n">
+        <x:v>2.2299999999999525</x:v>
+      </x:c>
+      <x:c r="L8" s="21" t="n">
+        <x:v>0.016717546900312342</x:v>
+      </x:c>
+      <x:c r="M8" s="21" t="n">
+        <x:v>0.17344054841769865</x:v>
+      </x:c>
+      <x:c r="N8" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>loiter_negative_disturbance</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>selected</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="21" t="n">
+        <x:v>5.541666666666667</x:v>
+      </x:c>
+      <x:c r="K9" s="21" t="n">
+        <x:v>0.42999999999999083</x:v>
+      </x:c>
+      <x:c r="L9" s="21" t="n">
+        <x:v>0.00864535302490578</x:v>
+      </x:c>
+      <x:c r="M9" s="21" t="n">
+        <x:v>0.12198570161509474</x:v>
+      </x:c>
+      <x:c r="N9" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O9" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>forward_1m</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>gain_zero_baseline</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O10" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>forward_1m</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>old_pr20_reference_0_1325</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D11" s="21" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E11" s="21" t="n">
+        <x:v>0.02999999999999936</x:v>
+      </x:c>
+      <x:c r="F11" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="21" t="n">
+        <x:v>58.791666666666664</x:v>
+      </x:c>
+      <x:c r="I11" s="21" t="n">
+        <x:v>0.20999999999999552</x:v>
+      </x:c>
+      <x:c r="J11" s="21" t="n">
+        <x:v>95.20833333333333</x:v>
+      </x:c>
+      <x:c r="K11" s="21" t="n">
+        <x:v>3.509999999999925</x:v>
+      </x:c>
+      <x:c r="L11" s="21" t="n">
+        <x:v>0.0144</x:v>
+      </x:c>
+      <x:c r="M11" s="21" t="n">
+        <x:v>0.1663289000505812</x:v>
+      </x:c>
+      <x:c r="N11" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>forward_1m</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>selected</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="21" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="I12" s="21" t="n">
+        <x:v>0.02999999999999936</x:v>
+      </x:c>
+      <x:c r="J12" s="21" t="n">
+        <x:v>4.291666666666667</x:v>
+      </x:c>
+      <x:c r="K12" s="21" t="n">
+        <x:v>0.1599999999999966</x:v>
+      </x:c>
+      <x:c r="L12" s="21" t="n">
+        <x:v>0.006095249493245699</x:v>
+      </x:c>
+      <x:c r="M12" s="21" t="n">
+        <x:v>0.08682762027868617</x:v>
+      </x:c>
+      <x:c r="N12" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O12" t="str"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>backward_1m</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>gain_zero_baseline</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>backward_1m</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>old_pr20_reference_0_1325</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="21" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E14" s="21" t="n">
+        <x:v>0.02999999999999936</x:v>
+      </x:c>
+      <x:c r="F14" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G14" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H14" s="21" t="n">
+        <x:v>58.791666666666664</x:v>
+      </x:c>
+      <x:c r="I14" s="21" t="n">
+        <x:v>0.20999999999999552</x:v>
+      </x:c>
+      <x:c r="J14" s="21" t="n">
+        <x:v>95.20833333333333</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="n">
+        <x:v>3.509999999999925</x:v>
+      </x:c>
+      <x:c r="L14" s="21" t="n">
+        <x:v>0.0144</x:v>
+      </x:c>
+      <x:c r="M14" s="21" t="n">
+        <x:v>0.1663289000505812</x:v>
+      </x:c>
+      <x:c r="N14" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>backward_1m</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>selected</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="21" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="I15" s="21" t="n">
+        <x:v>0.02999999999999936</x:v>
+      </x:c>
+      <x:c r="J15" s="21" t="n">
+        <x:v>4.291666666666667</x:v>
+      </x:c>
+      <x:c r="K15" s="21" t="n">
+        <x:v>0.1599999999999966</x:v>
+      </x:c>
+      <x:c r="L15" s="21" t="n">
+        <x:v>0.006095249493245699</x:v>
+      </x:c>
+      <x:c r="M15" s="21" t="n">
+        <x:v>0.08682762027868617</x:v>
+      </x:c>
+      <x:c r="N15" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O15" t="str"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>pitch_positive_recovery</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>gain_zero_baseline</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N16" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O16" t="str"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>pitch_positive_recovery</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>old_pr20_reference_0_1325</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D17" s="21" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E17" s="21" t="n">
+        <x:v>0.03999999999999915</x:v>
+      </x:c>
+      <x:c r="F17" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="21" t="n">
+        <x:v>62.18749999999999</x:v>
+      </x:c>
+      <x:c r="I17" s="21" t="n">
+        <x:v>0.2199999999999953</x:v>
+      </x:c>
+      <x:c r="J17" s="21" t="n">
+        <x:v>99.3125</x:v>
+      </x:c>
+      <x:c r="K17" s="21" t="n">
+        <x:v>4.519999999999904</x:v>
+      </x:c>
+      <x:c r="L17" s="21" t="n">
+        <x:v>0.016000000000000004</x:v>
+      </x:c>
+      <x:c r="M17" s="21" t="n">
+        <x:v>0.17252627253133182</x:v>
+      </x:c>
+      <x:c r="N17" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>pitch_positive_recovery</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>selected</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="21" t="n">
+        <x:v>0.375</x:v>
+      </x:c>
+      <x:c r="I18" s="21" t="n">
+        <x:v>0.02999999999999936</x:v>
+      </x:c>
+      <x:c r="J18" s="21" t="n">
+        <x:v>5.75</x:v>
+      </x:c>
+      <x:c r="K18" s="21" t="n">
+        <x:v>0.19499999999999584</x:v>
+      </x:c>
+      <x:c r="L18" s="21" t="n">
+        <x:v>0.007125651903882047</x:v>
+      </x:c>
+      <x:c r="M18" s="21" t="n">
+        <x:v>0.09625651903882049</x:v>
+      </x:c>
+      <x:c r="N18" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O18" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>pitch_negative_recovery</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>gain_zero_baseline</x:v>
+      </x:c>
+      <x:c r="C19" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O19" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>pitch_negative_recovery</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>old_pr20_reference_0_1325</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="21" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E20" s="21" t="n">
+        <x:v>0.03999999999999915</x:v>
+      </x:c>
+      <x:c r="F20" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="21" t="n">
+        <x:v>62.18749999999999</x:v>
+      </x:c>
+      <x:c r="I20" s="21" t="n">
+        <x:v>0.2199999999999953</x:v>
+      </x:c>
+      <x:c r="J20" s="21" t="n">
+        <x:v>99.3125</x:v>
+      </x:c>
+      <x:c r="K20" s="21" t="n">
+        <x:v>4.519999999999904</x:v>
+      </x:c>
+      <x:c r="L20" s="21" t="n">
+        <x:v>0.016000000000000004</x:v>
+      </x:c>
+      <x:c r="M20" s="21" t="n">
+        <x:v>0.17252627253133182</x:v>
+      </x:c>
+      <x:c r="N20" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O20" t="str">
+        <x:v>excessive_moving_mass_rate_limiter_duty; excessive_moving_mass_acceleration_limiter_duty; excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>pitch_negative_recovery</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>selected</x:v>
+      </x:c>
+      <x:c r="C21" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G21" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="21" t="n">
+        <x:v>0.375</x:v>
+      </x:c>
+      <x:c r="I21" s="21" t="n">
+        <x:v>0.02999999999999936</x:v>
+      </x:c>
+      <x:c r="J21" s="21" t="n">
+        <x:v>5.75</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="n">
+        <x:v>0.19499999999999584</x:v>
+      </x:c>
+      <x:c r="L21" s="21" t="n">
+        <x:v>0.007125651903882047</x:v>
+      </x:c>
+      <x:c r="M21" s="21" t="n">
+        <x:v>0.09625651903882049</x:v>
+      </x:c>
+      <x:c r="N21" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O21" t="str"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>stick_release</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>gain_zero_baseline</x:v>
+      </x:c>
+      <x:c r="C22" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O22" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>stick_release</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>old_pr20_reference_0_1325</x:v>
+      </x:c>
+      <x:c r="C23" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G23" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J23" s="21" t="n">
+        <x:v>5.583333333333333</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="n">
+        <x:v>0.1499999999999968</x:v>
+      </x:c>
+      <x:c r="L23" s="21" t="n">
+        <x:v>0.004884548147316462</x:v>
+      </x:c>
+      <x:c r="M23" s="21" t="n">
+        <x:v>0.08834552429166276</x:v>
+      </x:c>
+      <x:c r="N23" s="21" t="n">
+        <x:v>1.0000000000000222</x:v>
+      </x:c>
+      <x:c r="O23" t="str"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>stick_release</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>selected</x:v>
+      </x:c>
+      <x:c r="C24" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D24" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J24" s="21" t="n">
+        <x:v>3.0833333333333335</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="n">
+        <x:v>0.05999999999999872</x:v>
+      </x:c>
+      <x:c r="L24" s="21" t="n">
+        <x:v>0.0020188811768735945</x:v>
+      </x:c>
+      <x:c r="M24" s="21" t="n">
+        <x:v>0.043757472028742556</x:v>
+      </x:c>
+      <x:c r="N24" s="21" t="n">
+        <x:v>1.0000000000000215</x:v>
+      </x:c>
+      <x:c r="O24" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde37cd326fe24920"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3668,37 +5858,53 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>moving_mass_acceleration_limit</x:v>
+        <x:v>excessive_moving_mass_acceleration_limiter_continuous_duration</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>29</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>moving_mass_saturation</x:v>
+        <x:v>excessive_moving_mass_acceleration_limiter_duty</x:v>
       </x:c>
       <x:c r="B3" t="n">
-        <x:v>29</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
+        <x:v>excessive_moving_mass_rate_limiter_duty</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>premature_pause</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
         <x:v>second_acceleration_lobe_after_full_pause</x:v>
       </x:c>
-      <x:c r="B4" t="n">
+      <x:c r="B6" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R587a117e126b4624"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c4147711fa47b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3720,50 +5926,50 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="24" t="str">
+      <x:c r="A4" s="23" t="str">
         <x:v>Stage 1</x:v>
       </x:c>
-      <x:c r="B4" s="24" t="str">
+      <x:c r="B4" s="23" t="str">
         <x:v>0.000..0.200 m/Nm at 0.025 plus old PR #20 gain 0.1325.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="24" t="str">
+      <x:c r="A5" s="23" t="str">
         <x:v>Stage 2</x:v>
       </x:c>
-      <x:c r="B5" s="24" t="str">
+      <x:c r="B5" s="23" t="str">
         <x:v>Best valid Stage-1 gain ±0.025 at 0.0025.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="24" t="str">
+      <x:c r="A6" s="23" t="str">
         <x:v>Stage 3</x:v>
       </x:c>
-      <x:c r="B6" s="24" t="str">
+      <x:c r="B6" s="23" t="str">
         <x:v>Best valid Stage-2 gain ±0.005 at 0.0005; upper-bound extension only, never past 0.300 without authorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="24" t="str">
+      <x:c r="A7" s="23" t="str">
         <x:v>Selection</x:v>
       </x:c>
-      <x:c r="B7" s="24" t="str">
+      <x:c r="B7" s="23" t="str">
         <x:v>Valid raw aggregate score rank 1; no near-equivalent lower-effort tie-break. Gain 0 is accepted when it is rank 1.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="24" t="str">
+      <x:c r="A8" s="23" t="str">
         <x:v>Hard gates</x:v>
       </x:c>
-      <x:c r="B8" s="24" t="str">
+      <x:c r="B8" s="23" t="str">
         <x:v>Mirrored reversal, pause/lobe/capture/shaped-vx, finite/crash/ground, symmetry, vane and Moving-mass chatter/saturation, and physical limits.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="24" t="str">
+      <x:c r="A9" s="23" t="str">
         <x:v>PR #20</x:v>
       </x:c>
-      <x:c r="B9" s="24" t="str">
+      <x:c r="B9" s="23" t="str">
         <x:v>Read-only reference; obsolete pre-PR-22 Pitch controller; not cherry-picked or modified.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Clarify limiter gates in workbook
</commit_message>
<xml_diff>
--- a/results/analysis/moving_mass_gain_resweep/moving_mass_gain_resweep.xlsx
+++ b/results/analysis/moving_mass_gain_resweep/moving_mass_gain_resweep.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Reaaec09ab46b44dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gain Ranking" sheetId="2" r:id="Rdcbdd6cb606641b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="3" r:id="Rb2aabe9abcee4f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Gates" sheetId="4" r:id="R5936a19774b14f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limiter Diagnostics" sheetId="5" r:id="R6644eef6c0ec4b7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejections" sheetId="6" r:id="R8cef17b49d9a4878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="7" r:id="Reb5f0335af6a49bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R531a43d58aeb45c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gain Ranking" sheetId="2" r:id="R8979b208eac241ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="3" r:id="Rbc8c65b9f0524400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Gates" sheetId="4" r:id="Rbedb6941b9d14386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limiter Diagnostics" sheetId="5" r:id="R1e4f00cc4e554793"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejections" sheetId="6" r:id="Ref5f7be5edeb4db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="7" r:id="Re45fed9ec6684bde"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3063,7 +3063,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4866bf3b43fb446e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R646f5c3687da4197"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3487,7 +3487,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce24b851ab8f4183"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7fc011ec1ac42b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4788,7 +4788,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46afc51e2124966"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c1395ba2d064f16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5835,7 +5835,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde37cd326fe24920"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd57275dd31c54c00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5899,7 +5899,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c4147711fa47b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra64a65b98ce94048"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5954,22 +5954,30 @@
         <x:v>Selection</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
-        <x:v>Valid raw aggregate score rank 1; no near-equivalent lower-effort tie-break. Gain 0 is accepted when it is rank 1.</x:v>
+        <x:v>Valid raw aggregate score rank 1; no near-equivalent lower-effort tie-break. A nonzero result requires at least 1% improvement.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="23" t="str">
-        <x:v>Hard gates</x:v>
+        <x:v>Limiter gates</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Mirrored reversal, pause/lobe/capture/shaped-vx, finite/crash/ground, symmetry, vane and Moving-mass chatter/saturation, and physical limits.</x:v>
+        <x:v>Clip/rail &gt;5% or &gt;0.5 s; rate &gt;20% or &gt;1.0 s; acceleration &gt;30% or &gt;1.0 s. Actual physical violations require max + 1e-9.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="23" t="str">
+        <x:v>Other hard gates</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>Mirrored reversal, pause/lobe/capture/shaped-vx, finite/crash/ground, symmetry, Moving-mass chatter, and vane/servo/mixer saturation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="23" t="str">
         <x:v>PR #20</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="str">
+      <x:c r="B10" s="23" t="str">
         <x:v>Read-only reference; obsolete pre-PR-22 Pitch controller; not cherry-picked or modified.</x:v>
       </x:c>
     </x:row>

</xml_diff>